<commit_message>
feat: Add expected predicted price to Monte Carlo dashboard
</commit_message>
<xml_diff>
--- a/backend/outputs/MSFT_Financial_Model.xlsx
+++ b/backend/outputs/MSFT_Financial_Model.xlsx
@@ -11,14 +11,19 @@
     <sheet name="Raw Balance Sheet" sheetId="2" r:id="rId2"/>
     <sheet name="Cash Flow Statement" sheetId="3" r:id="rId3"/>
     <sheet name="Ratio Analysis" sheetId="4" r:id="rId4"/>
-    <sheet name="Summary Dashboard" sheetId="5" r:id="rId5"/>
+    <sheet name="Assumptions &amp; Drivers" sheetId="5" r:id="rId5"/>
+    <sheet name="CapEx &amp; Depreciation" sheetId="6" r:id="rId6"/>
+    <sheet name="OpEx &amp; R&amp;D Budget" sheetId="7" r:id="rId7"/>
+    <sheet name="Valuation &amp; Returns" sheetId="8" r:id="rId8"/>
+    <sheet name="Sensitivity Analysis" sheetId="9" r:id="rId9"/>
+    <sheet name="Summary Dashboard" sheetId="10" r:id="rId10"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="470" uniqueCount="278">
   <si>
     <t>Tax Effect Of Unusual Items</t>
   </si>
@@ -587,49 +592,232 @@
     <t>Net Income From Continuing Operations</t>
   </si>
   <si>
+    <t>Gross Profit Margin (%)</t>
+  </si>
+  <si>
+    <t>EBITDA Margin (%)</t>
+  </si>
+  <si>
+    <t>EBIT Margin (%)</t>
+  </si>
+  <si>
+    <t>Net Profit Margin (%)</t>
+  </si>
+  <si>
+    <t>Interest Coverage Ratio</t>
+  </si>
+  <si>
+    <t>Cash Conversion Ratio</t>
+  </si>
+  <si>
+    <t>Asset Turnover</t>
+  </si>
+  <si>
+    <t>Asset to Equity</t>
+  </si>
+  <si>
+    <t>Return on Equity (ROE) (%)</t>
+  </si>
+  <si>
+    <t>Debt to Equity</t>
+  </si>
+  <si>
+    <t>Return on Assets (ROA) (%)</t>
+  </si>
+  <si>
+    <t>Current Ratio</t>
+  </si>
+  <si>
+    <t>Quick Ratio</t>
+  </si>
+  <si>
+    <t>Debt to Capital</t>
+  </si>
+  <si>
+    <t>Inventory Days</t>
+  </si>
+  <si>
+    <t>Receivable Days</t>
+  </si>
+  <si>
+    <t>Payable Days</t>
+  </si>
+  <si>
+    <t>Cash to Debt</t>
+  </si>
+  <si>
     <t>Revenue Growth (%)</t>
   </si>
   <si>
-    <t>Gross Profit Margin (%)</t>
-  </si>
-  <si>
-    <t>EBITDA Margin (%)</t>
-  </si>
-  <si>
-    <t>EBIT Margin (%)</t>
-  </si>
-  <si>
-    <t>Net Profit Margin (%)</t>
-  </si>
-  <si>
-    <t>Debt to Equity</t>
-  </si>
-  <si>
-    <t>Interest Coverage Ratio</t>
-  </si>
-  <si>
-    <t>Debt to EBITDA</t>
-  </si>
-  <si>
-    <t>Asset Turnover</t>
-  </si>
-  <si>
-    <t>Current Ratio</t>
-  </si>
-  <si>
-    <t>Quick Ratio</t>
-  </si>
-  <si>
-    <t>Return on Equity (ROE) (%)</t>
-  </si>
-  <si>
-    <t>Return on Assets (ROA) (%)</t>
-  </si>
-  <si>
-    <t>Return on Invested Capital (ROIC) (%)</t>
+    <t>Debt to Assets</t>
+  </si>
+  <si>
+    <t>% of Debt Change</t>
+  </si>
+  <si>
+    <t>FCFF</t>
   </si>
   <si>
     <t>Operating CF Ratio</t>
+  </si>
+  <si>
+    <t>FCF to Net Profit</t>
+  </si>
+  <si>
+    <t>Month 1</t>
+  </si>
+  <si>
+    <t>Month 2</t>
+  </si>
+  <si>
+    <t>Month 3</t>
+  </si>
+  <si>
+    <t>Month 4</t>
+  </si>
+  <si>
+    <t>Month 5</t>
+  </si>
+  <si>
+    <t>Month 6</t>
+  </si>
+  <si>
+    <t>Month 7</t>
+  </si>
+  <si>
+    <t>Month 8</t>
+  </si>
+  <si>
+    <t>Month 9</t>
+  </si>
+  <si>
+    <t>Month 10</t>
+  </si>
+  <si>
+    <t>Month 11</t>
+  </si>
+  <si>
+    <t>Month 12</t>
+  </si>
+  <si>
+    <t>Month 13</t>
+  </si>
+  <si>
+    <t>Month 14</t>
+  </si>
+  <si>
+    <t>Month 15</t>
+  </si>
+  <si>
+    <t>Month 16</t>
+  </si>
+  <si>
+    <t>Month 17</t>
+  </si>
+  <si>
+    <t>Month 18</t>
+  </si>
+  <si>
+    <t>Month 19</t>
+  </si>
+  <si>
+    <t>Month 20</t>
+  </si>
+  <si>
+    <t>Month 21</t>
+  </si>
+  <si>
+    <t>Month 22</t>
+  </si>
+  <si>
+    <t>Month 23</t>
+  </si>
+  <si>
+    <t>Month 24</t>
+  </si>
+  <si>
+    <t>TAM (Total Addressable Market)</t>
+  </si>
+  <si>
+    <t>SAM (Serviceable Available Market)</t>
+  </si>
+  <si>
+    <t>SOM (Serviceable Obtainable Market)</t>
+  </si>
+  <si>
+    <t>Target Unit Price</t>
+  </si>
+  <si>
+    <t>New Customers/Month</t>
+  </si>
+  <si>
+    <t>Infrastructure (Labs)</t>
+  </si>
+  <si>
+    <t>Machinery &amp; Eqpt</t>
+  </si>
+  <si>
+    <t>Total CapEx</t>
+  </si>
+  <si>
+    <t>Depreciation Expense</t>
+  </si>
+  <si>
+    <t>Personnel (Sci/Eng)</t>
+  </si>
+  <si>
+    <t>Prototyping &amp; Materials</t>
+  </si>
+  <si>
+    <t>Testing &amp; Energy</t>
+  </si>
+  <si>
+    <t>COGS (BOM+Labor)</t>
+  </si>
+  <si>
+    <t>SG&amp;A (Legal/Marketing)</t>
+  </si>
+  <si>
+    <t>Total OpEx</t>
+  </si>
+  <si>
+    <t>Revenue</t>
+  </si>
+  <si>
+    <t>Op Cash Flow</t>
+  </si>
+  <si>
+    <t>Ending Cash Balance</t>
+  </si>
+  <si>
+    <t>Monthly Burn Rate</t>
+  </si>
+  <si>
+    <t>Runway (Months)</t>
+  </si>
+  <si>
+    <t>Discounted FCF</t>
+  </si>
+  <si>
+    <t>Best Case</t>
+  </si>
+  <si>
+    <t>Base Case</t>
+  </si>
+  <si>
+    <t>Worst Case</t>
+  </si>
+  <si>
+    <t>Cumulative 24M FCF</t>
+  </si>
+  <si>
+    <t>NPV (15% WACC)</t>
+  </si>
+  <si>
+    <t>IRR (Estimate)</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
   <si>
     <t>MSFT Financial Summary Dashboard</t>
@@ -765,6 +953,942 @@
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Profitability Margins</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Gross Profit Margin (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="circle"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$2:$E$2</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>68.4016744842891</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>68.92008588349103</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>69.76444382797138</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>68.82374238616519</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>EBITDA Margin (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="circle"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$3:$E$3</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>50.55681646239976</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>49.61423212136942</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>54.26236731097168</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>56.85174142068124</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>EBIT Margin (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="circle"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$4:$E$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>43.26373127553336</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>43.07340207158531</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>45.17016016514226</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>44.72888358819269</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Net Profit Margin (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="circle"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$5:$E$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>36.68633681343622</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>34.14623787839464</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>35.95597294408498</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>36.14601524896707</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="50010001"/>
+        <c:axId val="50010002"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="50010001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50010002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50010001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Return on Assets &amp; Equity</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$12</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Return on Assets (ROA) (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$12:$E$12</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>19.93695866681285</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17.5643726819038</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>17.2085839859576</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>16.45097035070912</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Return on Equity (ROE) (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$10:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>43.67546925099975</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>35.08871464385641</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>32.82813797829981</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>29.64722734140952</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50020001"/>
+        <c:axId val="50020002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50020001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50020002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50020001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Liquidity Ratios (Current / Quick)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Current Ratio</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="diamond"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$13:$E$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1.784606970825182</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.76916725076573</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.274954903181521</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.353446444504242</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Quick Ratio</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:marker>
+            <c:symbol val="diamond"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$14:$E$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>1.745251467154666</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.745163179675273</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.265009657902719</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.346804231755159</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:marker val="1"/>
+        <c:axId val="50030001"/>
+        <c:axId val="50030002"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="50030001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50030002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50030002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50030001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Revenue YoY Growth</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$A$21</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Revenue Growth (%)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2563EB"/>
+            </a:solidFill>
+          </c:spPr>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Ratio Analysis'!$B$1:$E$1</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2022-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2023-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2024-06-30T00:00:00</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2025-06-30T00:00:00</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Ratio Analysis'!$B$21:$E$21</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>6.882029555656421</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>15.66996201307127</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>14.93215623240671</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50040001"/>
+        <c:axId val="50040002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50040001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50040002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50040002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorGridlines/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="50040001"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Chart 2"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>114300</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Chart 3"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>65</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 4"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1877,6 +3001,75 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="25.7109375" customWidth="1"/>
+    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="3" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>268</v>
+      </c>
+      <c r="B4" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>270</v>
+      </c>
+      <c r="B5" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>272</v>
+      </c>
+      <c r="B6" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" s="4" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>277</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F79"/>
@@ -4255,7 +5448,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -4281,16 +5474,16 @@
         <v>189</v>
       </c>
       <c r="B2" s="1">
-        <v>0</v>
+        <v>68.4016744842891</v>
       </c>
       <c r="C2" s="1">
-        <v>6.882029555656421</v>
+        <v>68.92008588349103</v>
       </c>
       <c r="D2" s="1">
-        <v>15.66996201307127</v>
+        <v>69.76444382797138</v>
       </c>
       <c r="E2" s="1">
-        <v>14.93215623240671</v>
+        <v>68.82374238616519</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -4298,16 +5491,16 @@
         <v>190</v>
       </c>
       <c r="B3" s="1">
-        <v>68.4016744842891</v>
+        <v>50.55681646239976</v>
       </c>
       <c r="C3" s="1">
-        <v>68.92008588349103</v>
+        <v>49.61423212136942</v>
       </c>
       <c r="D3" s="1">
-        <v>69.76444382797138</v>
+        <v>54.26236731097168</v>
       </c>
       <c r="E3" s="1">
-        <v>68.82374238616519</v>
+        <v>56.85174142068124</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -4315,16 +5508,16 @@
         <v>191</v>
       </c>
       <c r="B4" s="1">
-        <v>50.55681646239976</v>
+        <v>43.26373127553336</v>
       </c>
       <c r="C4" s="1">
-        <v>49.61423212136942</v>
+        <v>43.07340207158531</v>
       </c>
       <c r="D4" s="1">
-        <v>54.26236731097168</v>
+        <v>45.17016016514226</v>
       </c>
       <c r="E4" s="1">
-        <v>56.85174142068124</v>
+        <v>44.72888358819269</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -4332,16 +5525,16 @@
         <v>192</v>
       </c>
       <c r="B5" s="1">
-        <v>43.26373127553336</v>
+        <v>36.68633681343622</v>
       </c>
       <c r="C5" s="1">
-        <v>43.07340207158531</v>
+        <v>34.14623787839464</v>
       </c>
       <c r="D5" s="1">
-        <v>45.17016016514226</v>
+        <v>35.95597294408498</v>
       </c>
       <c r="E5" s="1">
-        <v>44.72888358819269</v>
+        <v>36.14601524896707</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -4349,16 +5542,16 @@
         <v>193</v>
       </c>
       <c r="B6" s="1">
-        <v>36.68633681343622</v>
+        <v>41.57973824527387</v>
       </c>
       <c r="C6" s="1">
-        <v>34.14623787839464</v>
+        <v>46.38160569105691</v>
       </c>
       <c r="D6" s="1">
-        <v>35.95597294408498</v>
+        <v>37.72470187393527</v>
       </c>
       <c r="E6" s="1">
-        <v>36.14601524896707</v>
+        <v>52.83522012578617</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4366,16 +5559,16 @@
         <v>194</v>
       </c>
       <c r="B7" s="1">
-        <v>0.3678951855988279</v>
+        <v>1.224050702521378</v>
       </c>
       <c r="C7" s="1">
-        <v>0.2907774593522546</v>
+        <v>1.210348115697683</v>
       </c>
       <c r="D7" s="1">
-        <v>0.2500288665323286</v>
+        <v>1.345057638195516</v>
       </c>
       <c r="E7" s="1">
-        <v>0.1763950634536609</v>
+        <v>1.33712389032917</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -4383,16 +5576,16 @@
         <v>195</v>
       </c>
       <c r="B8" s="1">
-        <v>41.57973824527387</v>
+        <v>0.5434437013485364</v>
       </c>
       <c r="C8" s="1">
-        <v>46.38160569105691</v>
+        <v>0.5143867603938094</v>
       </c>
       <c r="D8" s="1">
-        <v>37.72470187393527</v>
+        <v>0.4786015389631816</v>
       </c>
       <c r="E8" s="1">
-        <v>52.83522012578617</v>
+        <v>0.4551254194244616</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -4400,16 +5593,16 @@
         <v>196</v>
       </c>
       <c r="B9" s="1">
-        <v>0.6112391384590828</v>
+        <v>2.190678627613455</v>
       </c>
       <c r="C9" s="1">
-        <v>0.5703347917062964</v>
+        <v>1.997720913768105</v>
       </c>
       <c r="D9" s="1">
-        <v>0.5046801344269937</v>
+        <v>1.907660618972947</v>
       </c>
       <c r="E9" s="1">
-        <v>0.3782848937033684</v>
+        <v>1.802156754852553</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -4417,101 +5610,101 @@
         <v>197</v>
       </c>
       <c r="B10" s="1">
-        <v>0.5434437013485364</v>
+        <v>43.67546925099975</v>
       </c>
       <c r="C10" s="1">
-        <v>0.5143867603938094</v>
+        <v>35.08871464385641</v>
       </c>
       <c r="D10" s="1">
-        <v>0.4786015389631816</v>
+        <v>32.82813797829981</v>
       </c>
       <c r="E10" s="1">
-        <v>0.4551254194244616</v>
+        <v>29.64722734140952</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>57</v>
+        <v>198</v>
       </c>
       <c r="B11" s="1">
-        <v>74602000000</v>
+        <v>0.3678951855988279</v>
       </c>
       <c r="C11" s="1">
-        <v>80108000000</v>
+        <v>0.2907774593522546</v>
       </c>
       <c r="D11" s="1">
-        <v>34448000000</v>
+        <v>0.2500288665323286</v>
       </c>
       <c r="E11" s="1">
-        <v>49913000000</v>
+        <v>0.1763950634536609</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B12" s="1">
-        <v>1.784606970825182</v>
+        <v>19.93695866681285</v>
       </c>
       <c r="C12" s="1">
-        <v>1.76916725076573</v>
+        <v>17.5643726819038</v>
       </c>
       <c r="D12" s="1">
-        <v>1.274954903181521</v>
+        <v>17.2085839859576</v>
       </c>
       <c r="E12" s="1">
-        <v>1.353446444504242</v>
+        <v>16.45097035070912</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B13" s="1">
-        <v>1.745251467154666</v>
+        <v>1.784606970825182</v>
       </c>
       <c r="C13" s="1">
-        <v>1.745163179675273</v>
+        <v>1.76916725076573</v>
       </c>
       <c r="D13" s="1">
-        <v>1.265009657902719</v>
+        <v>1.274954903181521</v>
       </c>
       <c r="E13" s="1">
-        <v>1.346804231755159</v>
+        <v>1.353446444504242</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B14" s="1">
-        <v>43.67546925099975</v>
+        <v>1.745251467154666</v>
       </c>
       <c r="C14" s="1">
-        <v>35.08871464385641</v>
+        <v>1.745163179675273</v>
       </c>
       <c r="D14" s="1">
-        <v>32.82813797829981</v>
+        <v>1.265009657902719</v>
       </c>
       <c r="E14" s="1">
-        <v>29.64722734140952</v>
+        <v>1.346804231755159</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" t="s">
-        <v>201</v>
+        <v>57</v>
       </c>
       <c r="B15" s="1">
-        <v>19.93695866681285</v>
+        <v>74602000000</v>
       </c>
       <c r="C15" s="1">
-        <v>17.5643726819038</v>
+        <v>80108000000</v>
       </c>
       <c r="D15" s="1">
-        <v>17.2085839859576</v>
+        <v>34448000000</v>
       </c>
       <c r="E15" s="1">
-        <v>16.45097035070912</v>
+        <v>49913000000</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -4519,50 +5712,677 @@
         <v>202</v>
       </c>
       <c r="B16" s="1">
-        <v>32.71577919583682</v>
+        <v>0.2689498358295437</v>
       </c>
       <c r="C16" s="1">
-        <v>27.78318356012086</v>
+        <v>0.2252731152418591</v>
       </c>
       <c r="D16" s="1">
-        <v>26.97700580575731</v>
+        <v>0.2000184741540625</v>
       </c>
       <c r="E16" s="1">
-        <v>25.68795100574068</v>
+        <v>0.1499454298420806</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>130</v>
+        <v>203</v>
       </c>
       <c r="B17" s="1">
-        <v>65149000000</v>
+        <v>21.80095770151636</v>
       </c>
       <c r="C17" s="1">
-        <v>59475000000</v>
+        <v>13.85451619270303</v>
       </c>
       <c r="D17" s="1">
-        <v>74071000000</v>
+        <v>6.136357503305718</v>
       </c>
       <c r="E17" s="1">
-        <v>71611000000</v>
+        <v>3.898054217759106</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B18" s="1">
-        <v>0.9364022633095643</v>
+        <v>81.48113683361073</v>
       </c>
       <c r="C18" s="1">
-        <v>0.84092982169776</v>
+        <v>83.85966071302173</v>
       </c>
       <c r="D18" s="1">
-        <v>0.9462190508117427</v>
+        <v>84.76293437553545</v>
       </c>
       <c r="E18" s="1">
-        <v>0.9641971986573949</v>
+        <v>90.56851741420681</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>205</v>
+      </c>
+      <c r="B19" s="1">
+        <v>51.1355257336676</v>
+      </c>
+      <c r="C19" s="1">
+        <v>45.22139375017117</v>
+      </c>
+      <c r="D19" s="1">
+        <v>46.94832990269461</v>
+      </c>
+      <c r="E19" s="1">
+        <v>52.18991918222937</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>206</v>
+      </c>
+      <c r="B20" s="1">
+        <v>0.2273706544801697</v>
+      </c>
+      <c r="C20" s="1">
+        <v>0.5787375969315434</v>
+      </c>
+      <c r="D20" s="1">
+        <v>0.2728410326694177</v>
+      </c>
+      <c r="E20" s="1">
+        <v>0.4991417442397835</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21" s="1">
+        <v>0</v>
+      </c>
+      <c r="C21" s="1">
+        <v>6.882029555656421</v>
+      </c>
+      <c r="D21" s="1">
+        <v>15.66996201307127</v>
+      </c>
+      <c r="E21" s="1">
+        <v>14.93215623240671</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>208</v>
+      </c>
+      <c r="B22" s="1">
+        <v>0.1679366297555093</v>
+      </c>
+      <c r="C22" s="1">
+        <v>0.145554595413325</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.1310656958819751</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.0978799779645656</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>209</v>
+      </c>
+      <c r="B23" s="1">
+        <v>0</v>
+      </c>
+      <c r="C23" s="1">
+        <v>-2.129916761873674</v>
+      </c>
+      <c r="D23" s="1">
+        <v>11.9436337863754</v>
+      </c>
+      <c r="E23" s="1">
+        <v>-9.741236760171024</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>210</v>
+      </c>
+      <c r="B24" s="1">
+        <v>64658470901.61977</v>
+      </c>
+      <c r="C24" s="1">
+        <v>62097500655.01451</v>
+      </c>
+      <c r="D24" s="1">
+        <v>66521910564.35376</v>
+      </c>
+      <c r="E24" s="1">
+        <v>78748532990.36618</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>130</v>
+      </c>
+      <c r="B25" s="1">
+        <v>65149000000</v>
+      </c>
+      <c r="C25" s="1">
+        <v>59475000000</v>
+      </c>
+      <c r="D25" s="1">
+        <v>74071000000</v>
+      </c>
+      <c r="E25" s="1">
+        <v>71611000000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" t="s">
+        <v>211</v>
+      </c>
+      <c r="B26" s="1">
+        <v>0.8882271371422301</v>
+      </c>
+      <c r="C26" s="1">
+        <v>0.8330036142286475</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0.8912780338172605</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.8501357974588706</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" t="s">
+        <v>212</v>
+      </c>
+      <c r="B27" s="1">
+        <v>0.8956666391707223</v>
+      </c>
+      <c r="C27" s="1">
+        <v>0.8219206478627991</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.8404170826903876</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.7032268834943829</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Y6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="25" width="18.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25">
+      <c r="B1" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
+      <c r="A2" t="s">
+        <v>237</v>
+      </c>
+      <c r="B2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="C2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="D2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="E2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="F2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="G2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="H2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="I2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="J2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="K2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="L2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="M2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="N2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="O2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="P2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="R2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="S2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="T2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="U2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="V2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="W2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="X2" s="1">
+        <v>50000000000</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>50000000000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
+      <c r="A3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="C3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="D3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="E3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="F3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="G3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="H3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="I3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="J3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="K3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="L3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="M3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="N3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="O3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="P3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="R3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="S3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="T3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="U3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="V3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="W3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="X3" s="1">
+        <v>5000000000</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>5000000000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
+      <c r="A4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="C4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="D4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="E4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="F4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="G4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="H4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="I4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="J4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="K4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="L4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="M4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="N4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="O4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="P4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="R4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="S4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="T4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="U4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="V4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="W4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="X4" s="1">
+        <v>100000000</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>100000000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
+      <c r="A5" t="s">
+        <v>240</v>
+      </c>
+      <c r="B5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="C5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="D5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="E5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="F5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="G5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="I5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="J5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="K5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="L5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="M5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="N5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="O5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="P5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="R5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="S5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="T5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="U5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="V5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="W5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="X5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25">
+      <c r="A6" t="s">
+        <v>241</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+      <c r="F6" s="1">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
+        <v>0</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>0</v>
+      </c>
+      <c r="J6" s="1">
+        <v>0</v>
+      </c>
+      <c r="K6" s="1">
+        <v>0</v>
+      </c>
+      <c r="L6" s="1">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1">
+        <v>1</v>
+      </c>
+      <c r="N6" s="1">
+        <v>2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>2</v>
+      </c>
+      <c r="P6" s="1">
+        <v>3</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>3</v>
+      </c>
+      <c r="R6" s="1">
+        <v>5</v>
+      </c>
+      <c r="S6" s="1">
+        <v>5</v>
+      </c>
+      <c r="T6" s="1">
+        <v>8</v>
+      </c>
+      <c r="U6" s="1">
+        <v>10</v>
+      </c>
+      <c r="V6" s="1">
+        <v>12</v>
+      </c>
+      <c r="W6" s="1">
+        <v>15</v>
+      </c>
+      <c r="X6" s="1">
+        <v>20</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -4570,68 +6390,1870 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:Y5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25.7109375" customWidth="1"/>
-    <col min="2" max="2" width="40.7109375" customWidth="1"/>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="25" width="18.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="3" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+    <row r="1" spans="1:25">
+      <c r="B1" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
+      <c r="A2" t="s">
+        <v>242</v>
+      </c>
+      <c r="B2" s="1">
+        <v>2000000</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1">
+        <v>0</v>
+      </c>
+      <c r="S2" s="1">
+        <v>0</v>
+      </c>
+      <c r="T2" s="1">
+        <v>0</v>
+      </c>
+      <c r="U2" s="1">
+        <v>0</v>
+      </c>
+      <c r="V2" s="1">
+        <v>0</v>
+      </c>
+      <c r="W2" s="1">
+        <v>0</v>
+      </c>
+      <c r="X2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
+      <c r="A3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B3" s="1">
+        <v>5000000</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0</v>
+      </c>
+      <c r="F3" s="1">
+        <v>0</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>0</v>
+      </c>
+      <c r="J3" s="1">
+        <v>0</v>
+      </c>
+      <c r="K3" s="1">
+        <v>0</v>
+      </c>
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
+        <v>500000</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0</v>
+      </c>
+      <c r="R3" s="1">
+        <v>0</v>
+      </c>
+      <c r="S3" s="1">
+        <v>0</v>
+      </c>
+      <c r="T3" s="1">
+        <v>0</v>
+      </c>
+      <c r="U3" s="1">
+        <v>0</v>
+      </c>
+      <c r="V3" s="1">
+        <v>0</v>
+      </c>
+      <c r="W3" s="1">
+        <v>0</v>
+      </c>
+      <c r="X3" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
       <c r="A4" t="s">
-        <v>207</v>
-      </c>
-      <c r="B4" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
+        <v>244</v>
+      </c>
+      <c r="B4" s="1">
+        <v>7000000</v>
+      </c>
+      <c r="C4" s="1">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1">
+        <v>0</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0</v>
+      </c>
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0</v>
+      </c>
+      <c r="N4" s="1">
+        <v>500000</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0</v>
+      </c>
+      <c r="S4" s="1">
+        <v>0</v>
+      </c>
+      <c r="T4" s="1">
+        <v>0</v>
+      </c>
+      <c r="U4" s="1">
+        <v>0</v>
+      </c>
+      <c r="V4" s="1">
+        <v>0</v>
+      </c>
+      <c r="W4" s="1">
+        <v>0</v>
+      </c>
+      <c r="X4" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
       <c r="A5" t="s">
-        <v>209</v>
-      </c>
-      <c r="B5" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
+        <v>245</v>
+      </c>
+      <c r="B5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="C5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="D5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="E5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="F5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="G5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="H5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="I5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="J5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="K5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="L5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="M5" s="1">
+        <v>105000</v>
+      </c>
+      <c r="N5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="O5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="P5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="R5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="S5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="T5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="U5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="V5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="W5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="X5" s="1">
+        <v>112500</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>112500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Y7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="25" width="18.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25">
+      <c r="B1" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
+      <c r="A2" t="s">
+        <v>246</v>
+      </c>
+      <c r="B2" s="1">
+        <v>200000</v>
+      </c>
+      <c r="C2" s="1">
+        <v>210000</v>
+      </c>
+      <c r="D2" s="1">
+        <v>220000</v>
+      </c>
+      <c r="E2" s="1">
+        <v>230000</v>
+      </c>
+      <c r="F2" s="1">
+        <v>240000</v>
+      </c>
+      <c r="G2" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H2" s="1">
+        <v>260000</v>
+      </c>
+      <c r="I2" s="1">
+        <v>270000</v>
+      </c>
+      <c r="J2" s="1">
+        <v>280000</v>
+      </c>
+      <c r="K2" s="1">
+        <v>290000</v>
+      </c>
+      <c r="L2" s="1">
+        <v>300000</v>
+      </c>
+      <c r="M2" s="1">
+        <v>310000</v>
+      </c>
+      <c r="N2" s="1">
+        <v>320000</v>
+      </c>
+      <c r="O2" s="1">
+        <v>330000</v>
+      </c>
+      <c r="P2" s="1">
+        <v>340000</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>350000</v>
+      </c>
+      <c r="R2" s="1">
+        <v>360000</v>
+      </c>
+      <c r="S2" s="1">
+        <v>370000</v>
+      </c>
+      <c r="T2" s="1">
+        <v>380000</v>
+      </c>
+      <c r="U2" s="1">
+        <v>390000</v>
+      </c>
+      <c r="V2" s="1">
+        <v>400000</v>
+      </c>
+      <c r="W2" s="1">
+        <v>410000</v>
+      </c>
+      <c r="X2" s="1">
+        <v>420000</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>430000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
+      <c r="A3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="C3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="D3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="E3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="F3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="G3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="H3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="I3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="J3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="K3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="L3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="M3" s="1">
+        <v>150000</v>
+      </c>
+      <c r="N3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="O3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="P3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="R3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="S3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="T3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="U3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="V3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="W3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="X3" s="1">
+        <v>50000</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
+      <c r="A4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="C4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="D4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="E4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="F4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="G4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="H4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="I4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="J4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="K4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="L4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="M4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="N4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="O4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="P4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="R4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="S4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="T4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="U4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="V4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="W4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="X4" s="1">
+        <v>50000</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
+      <c r="A5" t="s">
+        <v>249</v>
+      </c>
+      <c r="B5" s="1">
+        <v>0</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0</v>
+      </c>
+      <c r="K5" s="1">
+        <v>0</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="M5" s="1">
+        <v>100000</v>
+      </c>
+      <c r="N5" s="1">
+        <v>200000</v>
+      </c>
+      <c r="O5" s="1">
+        <v>200000</v>
+      </c>
+      <c r="P5" s="1">
+        <v>300000</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>300000</v>
+      </c>
+      <c r="R5" s="1">
+        <v>500000</v>
+      </c>
+      <c r="S5" s="1">
+        <v>500000</v>
+      </c>
+      <c r="T5" s="1">
+        <v>800000</v>
+      </c>
+      <c r="U5" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="V5" s="1">
+        <v>1200000</v>
+      </c>
+      <c r="W5" s="1">
+        <v>1500000</v>
+      </c>
+      <c r="X5" s="1">
+        <v>2000000</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>2500000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25">
       <c r="A6" t="s">
-        <v>211</v>
-      </c>
-      <c r="B6" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
+        <v>250</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="C6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="D6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="E6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="F6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="G6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="H6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="I6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="J6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="K6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="L6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="M6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="N6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="O6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="P6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="R6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="S6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="T6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="U6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="V6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="W6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="X6" s="1">
+        <v>100000</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25">
       <c r="A7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B7" s="1">
+        <v>500000</v>
+      </c>
+      <c r="C7" s="1">
+        <v>510000</v>
+      </c>
+      <c r="D7" s="1">
+        <v>520000</v>
+      </c>
+      <c r="E7" s="1">
+        <v>530000</v>
+      </c>
+      <c r="F7" s="1">
+        <v>540000</v>
+      </c>
+      <c r="G7" s="1">
+        <v>550000</v>
+      </c>
+      <c r="H7" s="1">
+        <v>560000</v>
+      </c>
+      <c r="I7" s="1">
+        <v>570000</v>
+      </c>
+      <c r="J7" s="1">
+        <v>580000</v>
+      </c>
+      <c r="K7" s="1">
+        <v>590000</v>
+      </c>
+      <c r="L7" s="1">
+        <v>600000</v>
+      </c>
+      <c r="M7" s="1">
+        <v>710000</v>
+      </c>
+      <c r="N7" s="1">
+        <v>720000</v>
+      </c>
+      <c r="O7" s="1">
+        <v>730000</v>
+      </c>
+      <c r="P7" s="1">
+        <v>840000</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>850000</v>
+      </c>
+      <c r="R7" s="1">
+        <v>1060000</v>
+      </c>
+      <c r="S7" s="1">
+        <v>1070000</v>
+      </c>
+      <c r="T7" s="1">
+        <v>1380000</v>
+      </c>
+      <c r="U7" s="1">
+        <v>1590000</v>
+      </c>
+      <c r="V7" s="1">
+        <v>1800000</v>
+      </c>
+      <c r="W7" s="1">
+        <v>2110000</v>
+      </c>
+      <c r="X7" s="1">
+        <v>2620000</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>3130000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Y11"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="25" width="18.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:25">
+      <c r="B1" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C1" s="2" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" s="4" t="s">
+      <c r="D1" s="2" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="10" spans="1:2">
+      <c r="E1" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>232</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="Y1" s="2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
+      <c r="A2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
+      <c r="H2" s="1">
+        <v>0</v>
+      </c>
+      <c r="I2" s="1">
+        <v>0</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0</v>
+      </c>
+      <c r="K2" s="1">
+        <v>0</v>
+      </c>
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <v>250000</v>
+      </c>
+      <c r="N2" s="1">
+        <v>750000</v>
+      </c>
+      <c r="O2" s="1">
+        <v>1250000</v>
+      </c>
+      <c r="P2" s="1">
+        <v>2000000</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>2750000</v>
+      </c>
+      <c r="R2" s="1">
+        <v>4000000</v>
+      </c>
+      <c r="S2" s="1">
+        <v>5250000</v>
+      </c>
+      <c r="T2" s="1">
+        <v>7250000</v>
+      </c>
+      <c r="U2" s="1">
+        <v>9750000</v>
+      </c>
+      <c r="V2" s="1">
+        <v>12750000</v>
+      </c>
+      <c r="W2" s="1">
+        <v>16500000</v>
+      </c>
+      <c r="X2" s="1">
+        <v>21500000</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>27750000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="1">
+        <v>-500000</v>
+      </c>
+      <c r="C3" s="1">
+        <v>-510000</v>
+      </c>
+      <c r="D3" s="1">
+        <v>-520000</v>
+      </c>
+      <c r="E3" s="1">
+        <v>-530000</v>
+      </c>
+      <c r="F3" s="1">
+        <v>-540000</v>
+      </c>
+      <c r="G3" s="1">
+        <v>-550000</v>
+      </c>
+      <c r="H3" s="1">
+        <v>-560000</v>
+      </c>
+      <c r="I3" s="1">
+        <v>-570000</v>
+      </c>
+      <c r="J3" s="1">
+        <v>-580000</v>
+      </c>
+      <c r="K3" s="1">
+        <v>-590000</v>
+      </c>
+      <c r="L3" s="1">
+        <v>-600000</v>
+      </c>
+      <c r="M3" s="1">
+        <v>-460000</v>
+      </c>
+      <c r="N3" s="1">
+        <v>30000</v>
+      </c>
+      <c r="O3" s="1">
+        <v>520000</v>
+      </c>
+      <c r="P3" s="1">
+        <v>1160000</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>1900000</v>
+      </c>
+      <c r="R3" s="1">
+        <v>2940000</v>
+      </c>
+      <c r="S3" s="1">
+        <v>4180000</v>
+      </c>
+      <c r="T3" s="1">
+        <v>5870000</v>
+      </c>
+      <c r="U3" s="1">
+        <v>8160000</v>
+      </c>
+      <c r="V3" s="1">
+        <v>10950000</v>
+      </c>
+      <c r="W3" s="1">
+        <v>14390000</v>
+      </c>
+      <c r="X3" s="1">
+        <v>18880000</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>24620000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="1">
+        <v>-605000</v>
+      </c>
+      <c r="C4" s="1">
+        <v>-615000</v>
+      </c>
+      <c r="D4" s="1">
+        <v>-625000</v>
+      </c>
+      <c r="E4" s="1">
+        <v>-635000</v>
+      </c>
+      <c r="F4" s="1">
+        <v>-645000</v>
+      </c>
+      <c r="G4" s="1">
+        <v>-655000</v>
+      </c>
+      <c r="H4" s="1">
+        <v>-665000</v>
+      </c>
+      <c r="I4" s="1">
+        <v>-675000</v>
+      </c>
+      <c r="J4" s="1">
+        <v>-685000</v>
+      </c>
+      <c r="K4" s="1">
+        <v>-695000</v>
+      </c>
+      <c r="L4" s="1">
+        <v>-705000</v>
+      </c>
+      <c r="M4" s="1">
+        <v>-565000</v>
+      </c>
+      <c r="N4" s="1">
+        <v>-82500</v>
+      </c>
+      <c r="O4" s="1">
+        <v>407500</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1047500</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>1787500</v>
+      </c>
+      <c r="R4" s="1">
+        <v>2827500</v>
+      </c>
+      <c r="S4" s="1">
+        <v>4067500</v>
+      </c>
+      <c r="T4" s="1">
+        <v>5757500</v>
+      </c>
+      <c r="U4" s="1">
+        <v>8047500</v>
+      </c>
+      <c r="V4" s="1">
+        <v>10837500</v>
+      </c>
+      <c r="W4" s="1">
+        <v>14277500</v>
+      </c>
+      <c r="X4" s="1">
+        <v>18767500</v>
+      </c>
+      <c r="Y4" s="1">
+        <v>24507500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:25">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="1">
+        <v>-605000</v>
+      </c>
+      <c r="C5" s="1">
+        <v>-615000</v>
+      </c>
+      <c r="D5" s="1">
+        <v>-625000</v>
+      </c>
+      <c r="E5" s="1">
+        <v>-635000</v>
+      </c>
+      <c r="F5" s="1">
+        <v>-645000</v>
+      </c>
+      <c r="G5" s="1">
+        <v>-655000</v>
+      </c>
+      <c r="H5" s="1">
+        <v>-665000</v>
+      </c>
+      <c r="I5" s="1">
+        <v>-675000</v>
+      </c>
+      <c r="J5" s="1">
+        <v>-685000</v>
+      </c>
+      <c r="K5" s="1">
+        <v>-695000</v>
+      </c>
+      <c r="L5" s="1">
+        <v>-705000</v>
+      </c>
+      <c r="M5" s="1">
+        <v>-565000</v>
+      </c>
+      <c r="N5" s="1">
+        <v>-82500</v>
+      </c>
+      <c r="O5" s="1">
+        <v>407500</v>
+      </c>
+      <c r="P5" s="1">
+        <v>1047500</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>1787500</v>
+      </c>
+      <c r="R5" s="1">
+        <v>2827500</v>
+      </c>
+      <c r="S5" s="1">
+        <v>4067500</v>
+      </c>
+      <c r="T5" s="1">
+        <v>5757500</v>
+      </c>
+      <c r="U5" s="1">
+        <v>8047500</v>
+      </c>
+      <c r="V5" s="1">
+        <v>10837500</v>
+      </c>
+      <c r="W5" s="1">
+        <v>14277500</v>
+      </c>
+      <c r="X5" s="1">
+        <v>18767500</v>
+      </c>
+      <c r="Y5" s="1">
+        <v>24507500</v>
+      </c>
+    </row>
+    <row r="6" spans="1:25">
+      <c r="A6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B6" s="1">
+        <v>-500000</v>
+      </c>
+      <c r="C6" s="1">
+        <v>-510000</v>
+      </c>
+      <c r="D6" s="1">
+        <v>-520000</v>
+      </c>
+      <c r="E6" s="1">
+        <v>-530000</v>
+      </c>
+      <c r="F6" s="1">
+        <v>-540000</v>
+      </c>
+      <c r="G6" s="1">
+        <v>-550000</v>
+      </c>
+      <c r="H6" s="1">
+        <v>-560000</v>
+      </c>
+      <c r="I6" s="1">
+        <v>-570000</v>
+      </c>
+      <c r="J6" s="1">
+        <v>-580000</v>
+      </c>
+      <c r="K6" s="1">
+        <v>-590000</v>
+      </c>
+      <c r="L6" s="1">
+        <v>-600000</v>
+      </c>
+      <c r="M6" s="1">
+        <v>-460000</v>
+      </c>
+      <c r="N6" s="1">
+        <v>30000</v>
+      </c>
+      <c r="O6" s="1">
+        <v>520000</v>
+      </c>
+      <c r="P6" s="1">
+        <v>1160000</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>1900000</v>
+      </c>
+      <c r="R6" s="1">
+        <v>2940000</v>
+      </c>
+      <c r="S6" s="1">
+        <v>4180000</v>
+      </c>
+      <c r="T6" s="1">
+        <v>5870000</v>
+      </c>
+      <c r="U6" s="1">
+        <v>8160000</v>
+      </c>
+      <c r="V6" s="1">
+        <v>10950000</v>
+      </c>
+      <c r="W6" s="1">
+        <v>14390000</v>
+      </c>
+      <c r="X6" s="1">
+        <v>18880000</v>
+      </c>
+      <c r="Y6" s="1">
+        <v>24620000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25">
+      <c r="A7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="1">
+        <v>-7500000</v>
+      </c>
+      <c r="C7" s="1">
+        <v>-510000</v>
+      </c>
+      <c r="D7" s="1">
+        <v>-520000</v>
+      </c>
+      <c r="E7" s="1">
+        <v>-530000</v>
+      </c>
+      <c r="F7" s="1">
+        <v>-540000</v>
+      </c>
+      <c r="G7" s="1">
+        <v>-550000</v>
+      </c>
+      <c r="H7" s="1">
+        <v>-560000</v>
+      </c>
+      <c r="I7" s="1">
+        <v>-570000</v>
+      </c>
+      <c r="J7" s="1">
+        <v>-580000</v>
+      </c>
+      <c r="K7" s="1">
+        <v>-590000</v>
+      </c>
+      <c r="L7" s="1">
+        <v>-600000</v>
+      </c>
+      <c r="M7" s="1">
+        <v>-460000</v>
+      </c>
+      <c r="N7" s="1">
+        <v>-470000</v>
+      </c>
+      <c r="O7" s="1">
+        <v>520000</v>
+      </c>
+      <c r="P7" s="1">
+        <v>1160000</v>
+      </c>
+      <c r="Q7" s="1">
+        <v>1900000</v>
+      </c>
+      <c r="R7" s="1">
+        <v>2940000</v>
+      </c>
+      <c r="S7" s="1">
+        <v>4180000</v>
+      </c>
+      <c r="T7" s="1">
+        <v>5870000</v>
+      </c>
+      <c r="U7" s="1">
+        <v>8160000</v>
+      </c>
+      <c r="V7" s="1">
+        <v>10950000</v>
+      </c>
+      <c r="W7" s="1">
+        <v>14390000</v>
+      </c>
+      <c r="X7" s="1">
+        <v>18880000</v>
+      </c>
+      <c r="Y7" s="1">
+        <v>24620000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25">
+      <c r="A8" t="s">
+        <v>254</v>
+      </c>
+      <c r="B8" s="1">
+        <v>17500000</v>
+      </c>
+      <c r="C8" s="1">
+        <v>16990000</v>
+      </c>
+      <c r="D8" s="1">
+        <v>16470000</v>
+      </c>
+      <c r="E8" s="1">
+        <v>15940000</v>
+      </c>
+      <c r="F8" s="1">
+        <v>15400000</v>
+      </c>
+      <c r="G8" s="1">
+        <v>14850000</v>
+      </c>
+      <c r="H8" s="1">
+        <v>14290000</v>
+      </c>
+      <c r="I8" s="1">
+        <v>13720000</v>
+      </c>
+      <c r="J8" s="1">
+        <v>13140000</v>
+      </c>
+      <c r="K8" s="1">
+        <v>12550000</v>
+      </c>
+      <c r="L8" s="1">
+        <v>11950000</v>
+      </c>
+      <c r="M8" s="1">
+        <v>11490000</v>
+      </c>
+      <c r="N8" s="1">
+        <v>11020000</v>
+      </c>
+      <c r="O8" s="1">
+        <v>11540000</v>
+      </c>
+      <c r="P8" s="1">
+        <v>12700000</v>
+      </c>
+      <c r="Q8" s="1">
+        <v>14600000</v>
+      </c>
+      <c r="R8" s="1">
+        <v>17540000</v>
+      </c>
+      <c r="S8" s="1">
+        <v>21720000</v>
+      </c>
+      <c r="T8" s="1">
+        <v>27590000</v>
+      </c>
+      <c r="U8" s="1">
+        <v>35750000</v>
+      </c>
+      <c r="V8" s="1">
+        <v>46700000</v>
+      </c>
+      <c r="W8" s="1">
+        <v>61090000</v>
+      </c>
+      <c r="X8" s="1">
+        <v>79970000</v>
+      </c>
+      <c r="Y8" s="1">
+        <v>104590000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25">
+      <c r="A9" t="s">
+        <v>255</v>
+      </c>
+      <c r="B9" s="1">
+        <v>7500000</v>
+      </c>
+      <c r="C9" s="1">
+        <v>510000</v>
+      </c>
+      <c r="D9" s="1">
+        <v>520000</v>
+      </c>
+      <c r="E9" s="1">
+        <v>530000</v>
+      </c>
+      <c r="F9" s="1">
+        <v>540000</v>
+      </c>
+      <c r="G9" s="1">
+        <v>550000</v>
+      </c>
+      <c r="H9" s="1">
+        <v>560000</v>
+      </c>
+      <c r="I9" s="1">
+        <v>570000</v>
+      </c>
+      <c r="J9" s="1">
+        <v>580000</v>
+      </c>
+      <c r="K9" s="1">
+        <v>590000</v>
+      </c>
+      <c r="L9" s="1">
+        <v>600000</v>
+      </c>
+      <c r="M9" s="1">
+        <v>460000</v>
+      </c>
+      <c r="N9" s="1">
+        <v>470000</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>0</v>
+      </c>
+      <c r="R9" s="1">
+        <v>0</v>
+      </c>
+      <c r="S9" s="1">
+        <v>0</v>
+      </c>
+      <c r="T9" s="1">
+        <v>0</v>
+      </c>
+      <c r="U9" s="1">
+        <v>0</v>
+      </c>
+      <c r="V9" s="1">
+        <v>0</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0</v>
+      </c>
+      <c r="X9" s="1">
+        <v>0</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:25">
       <c r="A10" t="s">
-        <v>216</v>
+        <v>256</v>
+      </c>
+      <c r="B10" s="1">
+        <v>2.333333333333333</v>
+      </c>
+      <c r="C10" s="1">
+        <v>33.31372549019608</v>
+      </c>
+      <c r="D10" s="1">
+        <v>31.67307692307692</v>
+      </c>
+      <c r="E10" s="1">
+        <v>30.07547169811321</v>
+      </c>
+      <c r="F10" s="1">
+        <v>28.51851851851852</v>
+      </c>
+      <c r="G10" s="1">
+        <v>27</v>
+      </c>
+      <c r="H10" s="1">
+        <v>25.51785714285714</v>
+      </c>
+      <c r="I10" s="1">
+        <v>24.07017543859649</v>
+      </c>
+      <c r="J10" s="1">
+        <v>22.6551724137931</v>
+      </c>
+      <c r="K10" s="1">
+        <v>21.27118644067797</v>
+      </c>
+      <c r="L10" s="1">
+        <v>19.91666666666667</v>
+      </c>
+      <c r="M10" s="1">
+        <v>24.97826086956522</v>
+      </c>
+      <c r="N10" s="1">
+        <v>23.4468085106383</v>
+      </c>
+      <c r="O10" s="1">
+        <v>999</v>
+      </c>
+      <c r="P10" s="1">
+        <v>999</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>999</v>
+      </c>
+      <c r="R10" s="1">
+        <v>999</v>
+      </c>
+      <c r="S10" s="1">
+        <v>999</v>
+      </c>
+      <c r="T10" s="1">
+        <v>999</v>
+      </c>
+      <c r="U10" s="1">
+        <v>999</v>
+      </c>
+      <c r="V10" s="1">
+        <v>999</v>
+      </c>
+      <c r="W10" s="1">
+        <v>999</v>
+      </c>
+      <c r="X10" s="1">
+        <v>999</v>
+      </c>
+      <c r="Y10" s="1">
+        <v>999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25">
+      <c r="A11" t="s">
+        <v>257</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-7500000</v>
+      </c>
+      <c r="C11" s="1">
+        <v>-503703.7037037037</v>
+      </c>
+      <c r="D11" s="1">
+        <v>-507239.750038104</v>
+      </c>
+      <c r="E11" s="1">
+        <v>-510611.7141884048</v>
+      </c>
+      <c r="F11" s="1">
+        <v>-513823.1086172627</v>
+      </c>
+      <c r="G11" s="1">
+        <v>-516877.384068577</v>
+      </c>
+      <c r="H11" s="1">
+        <v>-519777.9305560551</v>
+      </c>
+      <c r="I11" s="1">
+        <v>-522528.078336775</v>
+      </c>
+      <c r="J11" s="1">
+        <v>-525131.0988699666</v>
+      </c>
+      <c r="K11" s="1">
+        <v>-527590.2057612266</v>
+      </c>
+      <c r="L11" s="1">
+        <v>-529908.5556923808</v>
+      </c>
+      <c r="M11" s="1">
+        <v>-401247.6306477287</v>
+      </c>
+      <c r="N11" s="1">
+        <v>-404909.042199533</v>
+      </c>
+      <c r="O11" s="1">
+        <v>442453.7997242073</v>
+      </c>
+      <c r="P11" s="1">
+        <v>974826.9851473514</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>1576987.034295418</v>
+      </c>
+      <c r="R11" s="1">
+        <v>2410054.25904017</v>
+      </c>
+      <c r="S11" s="1">
+        <v>3384236.769224124</v>
+      </c>
+      <c r="T11" s="1">
+        <v>4693831.847207895</v>
+      </c>
+      <c r="U11" s="1">
+        <v>6444430.626237856</v>
+      </c>
+      <c r="V11" s="1">
+        <v>8541093.604127878</v>
+      </c>
+      <c r="W11" s="1">
+        <v>11085751.12133944</v>
+      </c>
+      <c r="X11" s="1">
+        <v>14365187.15300499</v>
+      </c>
+      <c r="Y11" s="1">
+        <v>18501302.97692942</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="35.7109375" customWidth="1"/>
+    <col min="2" max="4" width="18.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="B1" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>261</v>
+      </c>
+      <c r="B2" s="1">
+        <v>104406000</v>
+      </c>
+      <c r="C2" s="1">
+        <v>79590000</v>
+      </c>
+      <c r="D2" s="1">
+        <v>52308000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B3" s="1">
+        <v>76617850.36567874</v>
+      </c>
+      <c r="C3" s="1">
+        <v>58936807.97359903</v>
+      </c>
+      <c r="D3" s="1">
+        <v>41255765.58151932</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>